<commit_message>
Refresh in-year data for August 2026
</commit_message>
<xml_diff>
--- a/docs/inyear.xlsx
+++ b/docs/inyear.xlsx
@@ -12,7 +12,7 @@
     <sheet name="By Area" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Club Health'!$A$1:$AC$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Club Health'!$A$1:$AA$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'By Area'!$A$1:$I$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,7 +495,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Program year 2026-2027. Dashboard snapshot 23-Aug-2026. Built 2026-08-24 14:37.</t>
+          <t>Program year 2026-2027. Dashboard snapshot 23-Aug-2026. Built 2026-08-24 21:39.</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC182"/>
+  <dimension ref="A1:AA182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -684,8 +684,6 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
-    <col width="13" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -824,16 +822,6 @@
           <t>Officer list on time (need 1)</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
-        <is>
-          <t>2025-2026 final</t>
-        </is>
-      </c>
-      <c r="AC1" s="3" t="inlineStr">
-        <is>
-          <t>2025-2026 status</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -931,10 +919,6 @@
       <c r="AA2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB2" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1032,14 +1016,6 @@
       <c r="AA3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB3" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC3" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1137,10 +1113,6 @@
       <c r="AA4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1238,14 +1210,6 @@
       <c r="AA5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB5" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC5" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1343,14 +1307,6 @@
       <c r="AA6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC6" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1448,14 +1404,6 @@
       <c r="AA7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB7" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC7" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1553,10 +1501,6 @@
       <c r="AA8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1654,14 +1598,6 @@
       <c r="AA9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB9" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC9" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1759,14 +1695,6 @@
       <c r="AA10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC10" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1864,10 +1792,6 @@
       <c r="AA11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB11" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1965,14 +1889,6 @@
       <c r="AA12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC12" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -2070,10 +1986,6 @@
       <c r="AA13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB13" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -2171,14 +2083,6 @@
       <c r="AA14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB14" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC14" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2276,10 +2180,6 @@
       <c r="AA15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2377,14 +2277,6 @@
       <c r="AA16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB16" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC16" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2482,14 +2374,6 @@
       <c r="AA17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB17" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC17" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2587,10 +2471,6 @@
       <c r="AA18" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2688,10 +2568,6 @@
       <c r="AA19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2789,14 +2665,6 @@
       <c r="AA20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB20" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC20" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2894,14 +2762,6 @@
       <c r="AA21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB21" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC21" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2999,10 +2859,6 @@
       <c r="AA22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB22" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -3100,10 +2956,6 @@
       <c r="AA23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB23" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -3201,14 +3053,6 @@
       <c r="AA24" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB24" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC24" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -3306,10 +3150,6 @@
       <c r="AA25" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -3407,14 +3247,6 @@
       <c r="AA26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB26" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC26" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3512,10 +3344,6 @@
       <c r="AA27" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB27" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -3613,10 +3441,6 @@
       <c r="AA28" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB28" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3714,14 +3538,6 @@
       <c r="AA29" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB29" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC29" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -3819,14 +3635,6 @@
       <c r="AA30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB30" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC30" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -3924,14 +3732,6 @@
       <c r="AA31" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB31" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC31" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -4029,10 +3829,6 @@
       <c r="AA32" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB32" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -4130,14 +3926,6 @@
       <c r="AA33" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB33" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC33" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -4235,10 +4023,6 @@
       <c r="AA34" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB34" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -4336,10 +4120,6 @@
       <c r="AA35" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB35" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -4437,14 +4217,6 @@
       <c r="AA36" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB36" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC36" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -4542,10 +4314,6 @@
       <c r="AA37" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -4643,14 +4411,6 @@
       <c r="AA38" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB38" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC38" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -4748,10 +4508,6 @@
       <c r="AA39" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB39" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -4849,10 +4605,6 @@
       <c r="AA40" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB40" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -4950,10 +4702,6 @@
       <c r="AA41" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB41" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -5051,10 +4799,6 @@
       <c r="AA42" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB42" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -5152,10 +4896,6 @@
       <c r="AA43" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB43" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -5253,10 +4993,6 @@
       <c r="AA44" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB44" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -5354,14 +5090,6 @@
       <c r="AA45" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB45" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC45" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -5459,10 +5187,6 @@
       <c r="AA46" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB46" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -5560,10 +5284,6 @@
       <c r="AA47" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB47" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -5661,14 +5381,6 @@
       <c r="AA48" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB48" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC48" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -5766,10 +5478,6 @@
       <c r="AA49" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB49" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -5867,14 +5575,6 @@
       <c r="AA50" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB50" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC50" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5972,14 +5672,6 @@
       <c r="AA51" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB51" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC51" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -6077,14 +5769,6 @@
       <c r="AA52" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB52" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC52" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -6182,14 +5866,6 @@
       <c r="AA53" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB53" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC53" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -6287,14 +5963,6 @@
       <c r="AA54" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB54" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC54" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -6392,10 +6060,6 @@
       <c r="AA55" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB55" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -6493,10 +6157,6 @@
       <c r="AA56" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB56" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -6594,14 +6254,6 @@
       <c r="AA57" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB57" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC57" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -6699,10 +6351,6 @@
       <c r="AA58" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB58" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -6800,10 +6448,6 @@
       <c r="AA59" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB59" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -6901,10 +6545,6 @@
       <c r="AA60" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB60" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -7002,10 +6642,6 @@
       <c r="AA61" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB61" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -7103,14 +6739,6 @@
       <c r="AA62" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB62" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC62" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -7208,10 +6836,6 @@
       <c r="AA63" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -7309,14 +6933,6 @@
       <c r="AA64" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB64" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC64" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -7414,14 +7030,6 @@
       <c r="AA65" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB65" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC65" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -7519,14 +7127,6 @@
       <c r="AA66" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB66" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC66" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -7624,10 +7224,6 @@
       <c r="AA67" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB67" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -7725,14 +7321,6 @@
       <c r="AA68" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB68" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC68" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -7830,14 +7418,6 @@
       <c r="AA69" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB69" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC69" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -7935,14 +7515,6 @@
       <c r="AA70" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB70" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC70" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -8040,8 +7612,6 @@
       <c r="AA71" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB71" s="4" t="n"/>
-      <c r="AC71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -8139,10 +7709,6 @@
       <c r="AA72" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB72" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -8240,10 +7806,6 @@
       <c r="AA73" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB73" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -8341,14 +7903,6 @@
       <c r="AA74" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB74" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC74" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -8446,10 +8000,6 @@
       <c r="AA75" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB75" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -8547,14 +8097,6 @@
       <c r="AA76" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB76" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC76" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -8652,10 +8194,6 @@
       <c r="AA77" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB77" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -8753,10 +8291,6 @@
       <c r="AA78" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB78" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -8854,10 +8388,6 @@
       <c r="AA79" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB79" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -8955,10 +8485,6 @@
       <c r="AA80" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB80" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -9056,14 +8582,6 @@
       <c r="AA81" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB81" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC81" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -9161,10 +8679,6 @@
       <c r="AA82" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB82" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -9262,14 +8776,6 @@
       <c r="AA83" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB83" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC83" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -9367,14 +8873,6 @@
       <c r="AA84" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB84" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC84" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -9472,10 +8970,6 @@
       <c r="AA85" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB85" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -9573,10 +9067,6 @@
       <c r="AA86" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB86" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -9674,10 +9164,6 @@
       <c r="AA87" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB87" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -9775,14 +9261,6 @@
       <c r="AA88" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB88" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC88" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -9880,10 +9358,6 @@
       <c r="AA89" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB89" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -9981,10 +9455,6 @@
       <c r="AA90" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB90" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -10082,14 +9552,6 @@
       <c r="AA91" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB91" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC91" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -10187,14 +9649,6 @@
       <c r="AA92" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB92" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC92" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -10292,14 +9746,6 @@
       <c r="AA93" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB93" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC93" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -10397,10 +9843,6 @@
       <c r="AA94" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB94" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -10498,10 +9940,6 @@
       <c r="AA95" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB95" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -10599,10 +10037,6 @@
       <c r="AA96" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB96" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -10700,10 +10134,6 @@
       <c r="AA97" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB97" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -10801,14 +10231,6 @@
       <c r="AA98" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB98" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC98" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -10906,14 +10328,6 @@
       <c r="AA99" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB99" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC99" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -11011,14 +10425,6 @@
       <c r="AA100" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB100" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC100" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -11116,10 +10522,6 @@
       <c r="AA101" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB101" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -11217,14 +10619,6 @@
       <c r="AA102" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB102" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC102" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -11322,14 +10716,6 @@
       <c r="AA103" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB103" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC103" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -11427,10 +10813,6 @@
       <c r="AA104" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB104" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -11528,10 +10910,6 @@
       <c r="AA105" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB105" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -11629,10 +11007,6 @@
       <c r="AA106" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB106" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -11730,14 +11104,6 @@
       <c r="AA107" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB107" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC107" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -11835,14 +11201,6 @@
       <c r="AA108" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB108" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC108" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -11940,10 +11298,6 @@
       <c r="AA109" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB109" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -12041,14 +11395,6 @@
       <c r="AA110" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB110" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC110" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -12146,10 +11492,6 @@
       <c r="AA111" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB111" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -12247,10 +11589,6 @@
       <c r="AA112" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB112" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -12348,14 +11686,6 @@
       <c r="AA113" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB113" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC113" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -12453,14 +11783,6 @@
       <c r="AA114" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB114" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC114" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -12558,10 +11880,6 @@
       <c r="AA115" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB115" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -12659,10 +11977,6 @@
       <c r="AA116" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB116" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -12760,14 +12074,6 @@
       <c r="AA117" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB117" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC117" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -12865,14 +12171,6 @@
       <c r="AA118" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB118" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC118" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -12970,10 +12268,6 @@
       <c r="AA119" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB119" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -13071,10 +12365,6 @@
       <c r="AA120" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB120" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -13172,10 +12462,6 @@
       <c r="AA121" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB121" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -13273,10 +12559,6 @@
       <c r="AA122" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB122" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -13374,10 +12656,6 @@
       <c r="AA123" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB123" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -13475,10 +12753,6 @@
       <c r="AA124" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB124" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -13576,14 +12850,6 @@
       <c r="AA125" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB125" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC125" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -13681,10 +12947,6 @@
       <c r="AA126" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB126" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -13782,10 +13044,6 @@
       <c r="AA127" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB127" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -13883,10 +13141,6 @@
       <c r="AA128" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB128" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -13984,14 +13238,6 @@
       <c r="AA129" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB129" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC129" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -14089,14 +13335,6 @@
       <c r="AA130" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB130" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC130" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -14194,10 +13432,6 @@
       <c r="AA131" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB131" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -14295,14 +13529,6 @@
       <c r="AA132" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB132" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC132" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -14400,14 +13626,6 @@
       <c r="AA133" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB133" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC133" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -14505,10 +13723,6 @@
       <c r="AA134" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB134" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -14606,14 +13820,6 @@
       <c r="AA135" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB135" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC135" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -14711,10 +13917,6 @@
       <c r="AA136" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB136" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -14812,10 +14014,6 @@
       <c r="AA137" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB137" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -14913,14 +14111,6 @@
       <c r="AA138" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB138" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC138" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -15018,10 +14208,6 @@
       <c r="AA139" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB139" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -15119,10 +14305,6 @@
       <c r="AA140" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB140" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -15220,14 +14402,6 @@
       <c r="AA141" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB141" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC141" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -15325,14 +14499,6 @@
       <c r="AA142" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB142" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC142" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -15430,14 +14596,6 @@
       <c r="AA143" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB143" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC143" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -15535,14 +14693,6 @@
       <c r="AA144" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB144" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC144" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -15640,14 +14790,6 @@
       <c r="AA145" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB145" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC145" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -15745,10 +14887,6 @@
       <c r="AA146" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB146" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC146" s="4" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -15846,14 +14984,6 @@
       <c r="AA147" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB147" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC147" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -15951,14 +15081,6 @@
       <c r="AA148" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB148" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC148" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -16056,10 +15178,6 @@
       <c r="AA149" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB149" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -16157,14 +15275,6 @@
       <c r="AA150" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB150" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC150" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -16262,14 +15372,6 @@
       <c r="AA151" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB151" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC151" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -16367,14 +15469,6 @@
       <c r="AA152" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB152" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="AC152" s="4" t="inlineStr">
-        <is>
-          <t>Select Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -16472,14 +15566,6 @@
       <c r="AA153" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB153" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC153" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -16577,14 +15663,6 @@
       <c r="AA154" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB154" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC154" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -16682,10 +15760,6 @@
       <c r="AA155" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB155" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -16783,14 +15857,6 @@
       <c r="AA156" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB156" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="AC156" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -16888,14 +15954,6 @@
       <c r="AA157" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB157" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC157" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -16993,10 +16051,6 @@
       <c r="AA158" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB158" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC158" s="4" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -17094,14 +16148,6 @@
       <c r="AA159" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB159" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC159" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -17199,14 +16245,6 @@
       <c r="AA160" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB160" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC160" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -17304,14 +16342,6 @@
       <c r="AA161" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB161" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC161" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -17409,10 +16439,6 @@
       <c r="AA162" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB162" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC162" s="4" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -17510,10 +16536,6 @@
       <c r="AA163" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB163" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -17611,10 +16633,6 @@
       <c r="AA164" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB164" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC164" s="4" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -17712,10 +16730,6 @@
       <c r="AA165" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB165" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC165" s="4" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -17813,14 +16827,6 @@
       <c r="AA166" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB166" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC166" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -17918,14 +16924,6 @@
       <c r="AA167" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB167" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC167" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -18023,10 +17021,6 @@
       <c r="AA168" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB168" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC168" s="4" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -18124,10 +17118,6 @@
       <c r="AA169" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB169" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -18225,10 +17215,6 @@
       <c r="AA170" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB170" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC170" s="4" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -18326,10 +17312,6 @@
       <c r="AA171" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB171" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -18427,10 +17409,6 @@
       <c r="AA172" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB172" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC172" s="4" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -18528,14 +17506,6 @@
       <c r="AA173" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB173" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC173" s="4" t="inlineStr">
-        <is>
-          <t>Smedley Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -18633,14 +17603,6 @@
       <c r="AA174" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB174" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC174" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -18738,10 +17700,6 @@
       <c r="AA175" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB175" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC175" s="4" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -18839,14 +17797,6 @@
       <c r="AA176" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB176" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC176" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -18944,14 +17894,6 @@
       <c r="AA177" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB177" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC177" s="4" t="inlineStr">
-        <is>
-          <t>President's Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -19049,14 +17991,6 @@
       <c r="AA178" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB178" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC178" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -19154,14 +18088,6 @@
       <c r="AA179" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB179" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC179" s="4" t="inlineStr">
-        <is>
-          <t>Distinguished</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -19259,10 +18185,6 @@
       <c r="AA180" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB180" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC180" s="4" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -19360,10 +18282,6 @@
       <c r="AA181" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AB181" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AC181" s="4" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -19461,13 +18379,9 @@
       <c r="AA182" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AB182" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AC182" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC182"/>
+  <autoFilter ref="A1:AA182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh in-year data for September 2026
</commit_message>
<xml_diff>
--- a/docs/inyear.xlsx
+++ b/docs/inyear.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -495,14 +495,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Program year 2026-2027. Dashboard snapshot 23-Aug-2026. Built 2026-08-24 18:50 PDT.</t>
+          <t>Program year 2026-2027. Dashboard snapshot 31-Aug-2026. Built 2026-09-01 12:07 PDT.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>310 days remain until 30 June 2027, when these scores become final.</t>
+          <t>302 days remain until 30 June 2027, when these scores become final.</t>
         </is>
       </c>
     </row>
@@ -574,70 +574,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officers trained Jun-Aug - closes 2026-08-31 (7 days) - 87 clubs short</t>
+          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (121 days) - 17 clubs short</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (129 days) - 17 clubs short</t>
+          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (180 days) - window opens 2026-11-01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (188 days) - window opens 2026-11-01</t>
+          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (211 days) - 98 clubs short</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (219 days) - 100 clubs short</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Membership rule</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Membership rule</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Distinguished also requires 20 members or a net growth of five over base.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Distinguished also requires 20 members or a net growth of five over base.</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Colour</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>Colour</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Green means the goal is met, pink means short, grey means the window has closed.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Green means the goal is met, pink means short, grey means the window has closed.</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Source: dashboards.toastmasters.org, read for each club individually.</t>
         </is>
@@ -883,11 +876,11 @@
         </is>
       </c>
       <c r="M2" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O2" s="7" t="inlineStr">
@@ -919,8 +912,8 @@
       <c r="W2" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X2" s="9" t="n">
-        <v>1</v>
+      <c r="X2" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y2" s="9" t="n">
         <v>0</v>
@@ -1126,7 +1119,7 @@
         <v>0</v>
       </c>
       <c r="X4" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y4" s="9" t="n">
         <v>0</v>
@@ -1162,7 +1155,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>10</v>
@@ -1205,8 +1198,8 @@
       <c r="P5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" s="9" t="n">
-        <v>1</v>
+      <c r="Q5" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="R5" s="9" t="n">
         <v>0</v>
@@ -1227,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="X5" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y5" s="9" t="n">
         <v>0</v>
@@ -1400,11 +1393,11 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O7" s="7" t="inlineStr">
@@ -1436,8 +1429,8 @@
       <c r="W7" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X7" s="9" t="n">
-        <v>3</v>
+      <c r="X7" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y7" s="9" t="n">
         <v>0</v>
@@ -1505,11 +1498,11 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr">
@@ -1541,8 +1534,8 @@
       <c r="W8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X8" s="9" t="n">
-        <v>1</v>
+      <c r="X8" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y8" s="9" t="n">
         <v>0</v>
@@ -1816,11 +1809,11 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1853,7 +1846,7 @@
         <v>0</v>
       </c>
       <c r="X11" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y11" s="9" t="n">
         <v>0</v>
@@ -1954,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="X12" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Y12" s="9" t="n">
         <v>0</v>
@@ -2022,11 +2015,11 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -2059,7 +2052,7 @@
         <v>0</v>
       </c>
       <c r="X13" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y13" s="9" t="n">
         <v>0</v>
@@ -2151,7 +2144,7 @@
         <v>1</v>
       </c>
       <c r="U14" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V14" s="9" t="n">
         <v>0</v>
@@ -2160,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y14" s="9" t="n">
         <v>0</v>
@@ -2228,11 +2221,11 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -2366,7 +2359,7 @@
         <v>0</v>
       </c>
       <c r="X16" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y16" s="9" t="n">
         <v>0</v>
@@ -2539,11 +2532,11 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O18" s="7" t="inlineStr">
@@ -2640,11 +2633,11 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -2846,11 +2839,11 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -2868,7 +2861,7 @@
         <v>0</v>
       </c>
       <c r="S21" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" s="9" t="n">
         <v>0</v>
@@ -2951,11 +2944,11 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -2988,7 +2981,7 @@
         <v>0</v>
       </c>
       <c r="X22" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y22" s="9" t="n">
         <v>0</v>
@@ -3059,9 +3052,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P23" s="9" t="n">
@@ -3396,7 +3389,7 @@
         <v>0</v>
       </c>
       <c r="X26" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y26" s="9" t="n">
         <v>0</v>
@@ -3464,11 +3457,11 @@
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3602,7 +3595,7 @@
         <v>0</v>
       </c>
       <c r="X28" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y28" s="9" t="n">
         <v>0</v>
@@ -3771,11 +3764,11 @@
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O30" s="7" t="inlineStr">
@@ -3807,8 +3800,8 @@
       <c r="W30" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X30" s="9" t="n">
-        <v>3</v>
+      <c r="X30" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y30" s="9" t="n">
         <v>0</v>
@@ -3981,11 +3974,11 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
@@ -4054,7 +4047,7 @@
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>10</v>
@@ -4089,9 +4082,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O33" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P33" s="9" t="n">
@@ -4106,8 +4099,8 @@
       <c r="S33" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T33" s="9" t="n">
-        <v>0</v>
+      <c r="T33" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U33" s="9" t="n">
         <v>0</v>
@@ -4288,11 +4281,11 @@
         </is>
       </c>
       <c r="M35" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
@@ -4325,7 +4318,7 @@
         <v>0</v>
       </c>
       <c r="X35" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y35" s="9" t="n">
         <v>0</v>
@@ -4494,11 +4487,11 @@
         </is>
       </c>
       <c r="M37" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N37" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
@@ -4707,9 +4700,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P39" s="9" t="n">
@@ -4737,7 +4730,7 @@
         <v>0</v>
       </c>
       <c r="X39" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y39" s="9" t="n">
         <v>0</v>
@@ -4801,11 +4794,11 @@
         </is>
       </c>
       <c r="M40" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O40" s="7" t="inlineStr">
@@ -4902,11 +4895,11 @@
         </is>
       </c>
       <c r="M41" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
@@ -5003,11 +4996,11 @@
         </is>
       </c>
       <c r="M42" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O42" s="7" t="inlineStr">
@@ -5039,8 +5032,8 @@
       <c r="W42" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X42" s="9" t="n">
-        <v>2</v>
+      <c r="X42" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y42" s="9" t="n">
         <v>0</v>
@@ -5104,11 +5097,11 @@
         </is>
       </c>
       <c r="M43" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
@@ -5120,7 +5113,7 @@
         <v>0</v>
       </c>
       <c r="Q43" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R43" s="9" t="n">
         <v>0</v>
@@ -5141,7 +5134,7 @@
         <v>0</v>
       </c>
       <c r="X43" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y43" s="9" t="n">
         <v>0</v>
@@ -5212,9 +5205,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O44" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P44" s="9" t="n">
@@ -5242,7 +5235,7 @@
         <v>0</v>
       </c>
       <c r="X44" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y44" s="9" t="n">
         <v>0</v>
@@ -5319,7 +5312,7 @@
         </is>
       </c>
       <c r="P45" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q45" s="9" t="n">
         <v>0</v>
@@ -5343,7 +5336,7 @@
         <v>0</v>
       </c>
       <c r="X45" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y45" s="9" t="n">
         <v>0</v>
@@ -5411,16 +5404,16 @@
         </is>
       </c>
       <c r="M46" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
-        </is>
-      </c>
-      <c r="O46" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+          <t>Officers trained Nov-Feb</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P46" s="9" t="n">
@@ -5512,11 +5505,11 @@
         </is>
       </c>
       <c r="M47" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
@@ -5650,7 +5643,7 @@
         <v>0</v>
       </c>
       <c r="X48" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y48" s="9" t="n">
         <v>0</v>
@@ -5704,13 +5697,13 @@
         </is>
       </c>
       <c r="I49" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
@@ -5718,11 +5711,11 @@
         </is>
       </c>
       <c r="M49" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N49" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O49" s="4" t="inlineStr">
@@ -5749,13 +5742,13 @@
         <v>0</v>
       </c>
       <c r="V49" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W49" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X49" s="9" t="n">
-        <v>1</v>
+      <c r="X49" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y49" s="9" t="n">
         <v>0</v>
@@ -5791,7 +5784,7 @@
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="6" t="n">
         <v>10</v>
@@ -5819,11 +5812,11 @@
         </is>
       </c>
       <c r="M50" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O50" s="4" t="inlineStr">
@@ -5843,8 +5836,8 @@
       <c r="S50" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="T50" s="9" t="n">
-        <v>0</v>
+      <c r="T50" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U50" s="9" t="n">
         <v>0</v>
@@ -5855,8 +5848,8 @@
       <c r="W50" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X50" s="9" t="n">
-        <v>2</v>
+      <c r="X50" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y50" s="9" t="n">
         <v>0</v>
@@ -5924,11 +5917,11 @@
         </is>
       </c>
       <c r="M51" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N51" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
@@ -5960,8 +5953,8 @@
       <c r="W51" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X51" s="9" t="n">
-        <v>1</v>
+      <c r="X51" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y51" s="9" t="n">
         <v>0</v>
@@ -6066,7 +6059,7 @@
         <v>0</v>
       </c>
       <c r="X52" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y52" s="9" t="n">
         <v>0</v>
@@ -6134,11 +6127,11 @@
         </is>
       </c>
       <c r="M53" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N53" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O53" s="7" t="inlineStr">
@@ -6171,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="X53" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y53" s="9" t="n">
         <v>0</v>
@@ -6252,7 +6245,7 @@
         </is>
       </c>
       <c r="P54" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q54" s="9" t="n">
         <v>1</v>
@@ -6276,7 +6269,7 @@
         <v>0</v>
       </c>
       <c r="X54" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y54" s="9" t="n">
         <v>0</v>
@@ -6344,11 +6337,11 @@
         </is>
       </c>
       <c r="M55" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N55" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O55" s="4" t="inlineStr">
@@ -6381,7 +6374,7 @@
         <v>0</v>
       </c>
       <c r="X55" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y55" s="9" t="n">
         <v>0</v>
@@ -6546,11 +6539,11 @@
         </is>
       </c>
       <c r="M57" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N57" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O57" s="4" t="inlineStr">
@@ -6559,7 +6552,7 @@
         </is>
       </c>
       <c r="P57" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q57" s="9" t="n">
         <v>0</v>
@@ -6582,8 +6575,8 @@
       <c r="W57" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X57" s="9" t="n">
-        <v>3</v>
+      <c r="X57" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y57" s="9" t="n">
         <v>0</v>
@@ -6789,7 +6782,7 @@
         <v>0</v>
       </c>
       <c r="X59" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y59" s="9" t="n">
         <v>0</v>
@@ -6853,11 +6846,11 @@
         </is>
       </c>
       <c r="M60" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O60" s="7" t="inlineStr">
@@ -6954,16 +6947,16 @@
         </is>
       </c>
       <c r="M61" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N61" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
-        </is>
-      </c>
-      <c r="O61" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+          <t>Officers trained Nov-Feb</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P61" s="9" t="n">
@@ -6990,8 +6983,8 @@
       <c r="W61" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X61" s="9" t="n">
-        <v>2</v>
+      <c r="X61" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y61" s="9" t="n">
         <v>0</v>
@@ -7092,7 +7085,7 @@
         <v>0</v>
       </c>
       <c r="X62" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y62" s="9" t="n">
         <v>0</v>
@@ -7160,11 +7153,11 @@
         </is>
       </c>
       <c r="M63" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N63" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O63" s="7" t="inlineStr">
@@ -7261,11 +7254,11 @@
         </is>
       </c>
       <c r="M64" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O64" s="7" t="inlineStr">
@@ -7297,8 +7290,8 @@
       <c r="W64" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X64" s="9" t="n">
-        <v>3</v>
+      <c r="X64" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y64" s="9" t="n">
         <v>0</v>
@@ -7576,11 +7569,11 @@
         </is>
       </c>
       <c r="M67" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N67" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O67" s="7" t="inlineStr">
@@ -7589,7 +7582,7 @@
         </is>
       </c>
       <c r="P67" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q67" s="9" t="n">
         <v>0</v>
@@ -7612,8 +7605,8 @@
       <c r="W67" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X67" s="9" t="n">
-        <v>3</v>
+      <c r="X67" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y67" s="9" t="n">
         <v>0</v>
@@ -7684,9 +7677,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O68" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O68" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P68" s="9" t="n">
@@ -7714,7 +7707,7 @@
         <v>0</v>
       </c>
       <c r="X68" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y68" s="9" t="n">
         <v>0</v>
@@ -7782,11 +7775,11 @@
         </is>
       </c>
       <c r="M69" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N69" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O69" s="7" t="inlineStr">
@@ -7924,7 +7917,7 @@
         <v>0</v>
       </c>
       <c r="X70" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Y70" s="9" t="n">
         <v>0</v>
@@ -7992,11 +7985,11 @@
         </is>
       </c>
       <c r="M71" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N71" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O71" s="7" t="inlineStr">
@@ -8028,8 +8021,8 @@
       <c r="W71" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X71" s="9" t="n">
-        <v>0</v>
+      <c r="X71" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y71" s="9" t="n">
         <v>0</v>
@@ -8164,7 +8157,7 @@
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F73" s="6" t="n">
         <v>10</v>
@@ -8192,11 +8185,11 @@
         </is>
       </c>
       <c r="M73" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N73" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O73" s="4" t="inlineStr">
@@ -8228,14 +8221,14 @@
       <c r="W73" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X73" s="9" t="n">
-        <v>3</v>
+      <c r="X73" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y73" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z73" s="9" t="n">
-        <v>0</v>
+      <c r="Z73" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA73" s="10" t="n">
         <v>1</v>
@@ -8435,7 +8428,7 @@
         <v>0</v>
       </c>
       <c r="X75" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y75" s="9" t="n">
         <v>0</v>
@@ -8499,11 +8492,11 @@
         </is>
       </c>
       <c r="M76" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O76" s="4" t="inlineStr">
@@ -8535,8 +8528,8 @@
       <c r="W76" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X76" s="9" t="n">
-        <v>0</v>
+      <c r="X76" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y76" s="9" t="n">
         <v>0</v>
@@ -8604,11 +8597,11 @@
         </is>
       </c>
       <c r="M77" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N77" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O77" s="7" t="inlineStr">
@@ -8705,11 +8698,11 @@
         </is>
       </c>
       <c r="M78" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O78" s="4" t="inlineStr">
@@ -8741,8 +8734,8 @@
       <c r="W78" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X78" s="9" t="n">
-        <v>3</v>
+      <c r="X78" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y78" s="9" t="n">
         <v>0</v>
@@ -8792,13 +8785,13 @@
         </is>
       </c>
       <c r="I79" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J79" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="7" t="inlineStr">
         <is>
@@ -8806,11 +8799,11 @@
         </is>
       </c>
       <c r="M79" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O79" s="4" t="inlineStr">
@@ -8837,13 +8830,13 @@
         <v>0</v>
       </c>
       <c r="V79" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W79" s="9" t="n">
         <v>0</v>
       </c>
       <c r="X79" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y79" s="9" t="n">
         <v>0</v>
@@ -8907,11 +8900,11 @@
         </is>
       </c>
       <c r="M80" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O80" s="4" t="inlineStr">
@@ -8943,8 +8936,8 @@
       <c r="W80" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X80" s="9" t="n">
-        <v>3</v>
+      <c r="X80" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y80" s="9" t="n">
         <v>0</v>
@@ -9045,7 +9038,7 @@
         <v>0</v>
       </c>
       <c r="X81" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y81" s="9" t="n">
         <v>0</v>
@@ -9150,7 +9143,7 @@
         <v>0</v>
       </c>
       <c r="X82" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Y82" s="9" t="n">
         <v>0</v>
@@ -9305,13 +9298,13 @@
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J84" s="4" t="n">
         <v>41</v>
       </c>
       <c r="K84" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L84" s="4" t="inlineStr">
         <is>
@@ -9319,11 +9312,11 @@
         </is>
       </c>
       <c r="M84" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N84" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O84" s="7" t="inlineStr">
@@ -9353,10 +9346,10 @@
         <v>4</v>
       </c>
       <c r="W84" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="X84" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="X84" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y84" s="9" t="n">
         <v>0</v>
@@ -9424,11 +9417,11 @@
         </is>
       </c>
       <c r="M85" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N85" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O85" s="7" t="inlineStr">
@@ -9562,7 +9555,7 @@
         <v>0</v>
       </c>
       <c r="X86" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y86" s="9" t="n">
         <v>0</v>
@@ -9663,7 +9656,7 @@
         <v>0</v>
       </c>
       <c r="X87" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y87" s="9" t="n">
         <v>0</v>
@@ -9734,9 +9727,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O88" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O88" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P88" s="9" t="n">
@@ -9764,7 +9757,7 @@
         <v>2</v>
       </c>
       <c r="X88" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y88" s="9" t="n">
         <v>0</v>
@@ -9832,11 +9825,11 @@
         </is>
       </c>
       <c r="M89" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N89" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O89" s="7" t="inlineStr">
@@ -9933,11 +9926,11 @@
         </is>
       </c>
       <c r="M90" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N90" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O90" s="7" t="inlineStr">
@@ -10071,7 +10064,7 @@
         <v>0</v>
       </c>
       <c r="X91" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y91" s="9" t="n">
         <v>0</v>
@@ -10176,7 +10169,7 @@
         <v>0</v>
       </c>
       <c r="X92" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y92" s="9" t="n">
         <v>0</v>
@@ -10251,9 +10244,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O93" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P93" s="9" t="n">
@@ -10281,7 +10274,7 @@
         <v>0</v>
       </c>
       <c r="X93" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y93" s="9" t="n">
         <v>0</v>
@@ -10450,11 +10443,11 @@
         </is>
       </c>
       <c r="M95" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N95" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O95" s="7" t="inlineStr">
@@ -10652,16 +10645,16 @@
         </is>
       </c>
       <c r="M97" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N97" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
-        </is>
-      </c>
-      <c r="O97" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+          <t>Officers trained Nov-Feb</t>
+        </is>
+      </c>
+      <c r="O97" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P97" s="9" t="n">
@@ -10790,7 +10783,7 @@
         <v>0</v>
       </c>
       <c r="X98" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y98" s="9" t="n">
         <v>0</v>
@@ -10858,11 +10851,11 @@
         </is>
       </c>
       <c r="M99" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N99" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O99" s="4" t="inlineStr">
@@ -10894,8 +10887,8 @@
       <c r="W99" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X99" s="9" t="n">
-        <v>3</v>
+      <c r="X99" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y99" s="9" t="n">
         <v>0</v>
@@ -11000,7 +10993,7 @@
         <v>0</v>
       </c>
       <c r="X100" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y100" s="9" t="n">
         <v>0</v>
@@ -11068,11 +11061,11 @@
         </is>
       </c>
       <c r="M101" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N101" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O101" s="7" t="inlineStr">
@@ -11155,13 +11148,13 @@
         </is>
       </c>
       <c r="I102" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J102" s="4" t="n">
         <v>40</v>
       </c>
       <c r="K102" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L102" s="4" t="inlineStr">
         <is>
@@ -11203,7 +11196,7 @@
         <v>4</v>
       </c>
       <c r="W102" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X102" s="10" t="n">
         <v>7</v>
@@ -11274,11 +11267,11 @@
         </is>
       </c>
       <c r="M103" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N103" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O103" s="4" t="inlineStr">
@@ -11379,11 +11372,11 @@
         </is>
       </c>
       <c r="M104" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N104" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O104" s="7" t="inlineStr">
@@ -11416,7 +11409,7 @@
         <v>0</v>
       </c>
       <c r="X104" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y104" s="9" t="n">
         <v>0</v>
@@ -11480,11 +11473,11 @@
         </is>
       </c>
       <c r="M105" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N105" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O105" s="4" t="inlineStr">
@@ -11517,7 +11510,7 @@
         <v>0</v>
       </c>
       <c r="X105" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y105" s="9" t="n">
         <v>0</v>
@@ -11581,11 +11574,11 @@
         </is>
       </c>
       <c r="M106" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N106" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O106" s="7" t="inlineStr">
@@ -11719,7 +11712,7 @@
         <v>0</v>
       </c>
       <c r="X107" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y107" s="9" t="n">
         <v>0</v>
@@ -11787,11 +11780,11 @@
         </is>
       </c>
       <c r="M108" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N108" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O108" s="7" t="inlineStr">
@@ -11824,7 +11817,7 @@
         <v>0</v>
       </c>
       <c r="X108" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y108" s="9" t="n">
         <v>0</v>
@@ -11892,11 +11885,11 @@
         </is>
       </c>
       <c r="M109" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N109" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O109" s="7" t="inlineStr">
@@ -11928,8 +11921,8 @@
       <c r="W109" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X109" s="9" t="n">
-        <v>0</v>
+      <c r="X109" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y109" s="9" t="n">
         <v>0</v>
@@ -12098,11 +12091,11 @@
         </is>
       </c>
       <c r="M111" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N111" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O111" s="7" t="inlineStr">
@@ -12199,11 +12192,11 @@
         </is>
       </c>
       <c r="M112" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N112" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O112" s="7" t="inlineStr">
@@ -12307,9 +12300,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O113" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O113" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P113" s="9" t="n">
@@ -12337,7 +12330,7 @@
         <v>0</v>
       </c>
       <c r="X113" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y113" s="9" t="n">
         <v>0</v>
@@ -12427,7 +12420,7 @@
         <v>0</v>
       </c>
       <c r="S114" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T114" s="10" t="n">
         <v>1</v>
@@ -12611,11 +12604,11 @@
         </is>
       </c>
       <c r="M116" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N116" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O116" s="7" t="inlineStr">
@@ -12647,8 +12640,8 @@
       <c r="W116" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X116" s="9" t="n">
-        <v>3</v>
+      <c r="X116" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y116" s="9" t="n">
         <v>0</v>
@@ -12749,7 +12742,7 @@
         <v>0</v>
       </c>
       <c r="X117" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y117" s="9" t="n">
         <v>0</v>
@@ -12929,13 +12922,13 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O119" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O119" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P119" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q119" s="9" t="n">
         <v>0</v>
@@ -12959,7 +12952,7 @@
         <v>0</v>
       </c>
       <c r="X119" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y119" s="9" t="n">
         <v>0</v>
@@ -13124,11 +13117,11 @@
         </is>
       </c>
       <c r="M121" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N121" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O121" s="7" t="inlineStr">
@@ -13427,11 +13420,11 @@
         </is>
       </c>
       <c r="M124" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N124" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O124" s="7" t="inlineStr">
@@ -13633,11 +13626,11 @@
         </is>
       </c>
       <c r="M126" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N126" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O126" s="7" t="inlineStr">
@@ -13669,8 +13662,8 @@
       <c r="W126" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X126" s="9" t="n">
-        <v>2</v>
+      <c r="X126" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y126" s="9" t="n">
         <v>0</v>
@@ -13734,11 +13727,11 @@
         </is>
       </c>
       <c r="M127" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N127" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O127" s="4" t="inlineStr">
@@ -14146,11 +14139,11 @@
         </is>
       </c>
       <c r="M131" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N131" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O131" s="7" t="inlineStr">
@@ -14284,7 +14277,7 @@
         <v>0</v>
       </c>
       <c r="X132" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y132" s="9" t="n">
         <v>0</v>
@@ -14338,13 +14331,13 @@
         </is>
       </c>
       <c r="I133" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J133" s="4" t="n">
         <v>24</v>
       </c>
       <c r="K133" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L133" s="4" t="inlineStr">
         <is>
@@ -14383,7 +14376,7 @@
         <v>0</v>
       </c>
       <c r="V133" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W133" s="9" t="n">
         <v>0</v>
@@ -14457,11 +14450,11 @@
         </is>
       </c>
       <c r="M134" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N134" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O134" s="7" t="inlineStr">
@@ -14595,7 +14588,7 @@
         <v>0</v>
       </c>
       <c r="X135" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y135" s="9" t="n">
         <v>0</v>
@@ -14663,11 +14656,11 @@
         </is>
       </c>
       <c r="M136" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N136" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O136" s="7" t="inlineStr">
@@ -14700,7 +14693,7 @@
         <v>0</v>
       </c>
       <c r="X136" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y136" s="9" t="n">
         <v>0</v>
@@ -14764,11 +14757,11 @@
         </is>
       </c>
       <c r="M137" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N137" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O137" s="7" t="inlineStr">
@@ -14970,11 +14963,11 @@
         </is>
       </c>
       <c r="M139" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N139" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O139" s="7" t="inlineStr">
@@ -15007,7 +15000,7 @@
         <v>0</v>
       </c>
       <c r="X139" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y139" s="9" t="n">
         <v>0</v>
@@ -15071,11 +15064,11 @@
         </is>
       </c>
       <c r="M140" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N140" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O140" s="7" t="inlineStr">
@@ -15107,8 +15100,8 @@
       <c r="W140" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X140" s="9" t="n">
-        <v>2</v>
+      <c r="X140" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y140" s="9" t="n">
         <v>0</v>
@@ -15249,7 +15242,7 @@
         </is>
       </c>
       <c r="E142" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F142" s="6" t="n">
         <v>10</v>
@@ -15295,8 +15288,8 @@
       <c r="Q142" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="R142" s="9" t="n">
-        <v>0</v>
+      <c r="R142" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="S142" s="10" t="n">
         <v>2</v>
@@ -15629,7 +15622,7 @@
         <v>0</v>
       </c>
       <c r="X145" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y145" s="9" t="n">
         <v>0</v>
@@ -15697,11 +15690,11 @@
         </is>
       </c>
       <c r="M146" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N146" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O146" s="7" t="inlineStr">
@@ -15734,7 +15727,7 @@
         <v>0</v>
       </c>
       <c r="X146" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y146" s="9" t="n">
         <v>0</v>
@@ -15798,11 +15791,11 @@
         </is>
       </c>
       <c r="M147" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N147" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O147" s="4" t="inlineStr">
@@ -15834,8 +15827,8 @@
       <c r="W147" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X147" s="9" t="n">
-        <v>1</v>
+      <c r="X147" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y147" s="9" t="n">
         <v>0</v>
@@ -15903,11 +15896,11 @@
         </is>
       </c>
       <c r="M148" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N148" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O148" s="4" t="inlineStr">
@@ -15940,7 +15933,7 @@
         <v>0</v>
       </c>
       <c r="X148" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y148" s="9" t="n">
         <v>0</v>
@@ -16045,7 +16038,7 @@
         <v>0</v>
       </c>
       <c r="X149" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y149" s="9" t="n">
         <v>0</v>
@@ -16081,7 +16074,7 @@
         </is>
       </c>
       <c r="E150" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F150" s="6" t="n">
         <v>10</v>
@@ -16124,8 +16117,8 @@
       <c r="P150" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q150" s="9" t="n">
-        <v>1</v>
+      <c r="Q150" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="R150" s="9" t="n">
         <v>0</v>
@@ -16230,7 +16223,7 @@
         <v>0</v>
       </c>
       <c r="Q151" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R151" s="9" t="n">
         <v>0</v>
@@ -16251,7 +16244,7 @@
         <v>0</v>
       </c>
       <c r="X151" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y151" s="9" t="n">
         <v>0</v>
@@ -16356,7 +16349,7 @@
         <v>0</v>
       </c>
       <c r="X152" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y152" s="9" t="n">
         <v>0</v>
@@ -16424,11 +16417,11 @@
         </is>
       </c>
       <c r="M153" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N153" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O153" s="4" t="inlineStr">
@@ -16460,8 +16453,8 @@
       <c r="W153" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X153" s="9" t="n">
-        <v>2</v>
+      <c r="X153" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y153" s="9" t="n">
         <v>0</v>
@@ -16501,7 +16494,7 @@
         </is>
       </c>
       <c r="E154" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F154" s="6" t="n">
         <v>10</v>
@@ -16515,13 +16508,13 @@
         </is>
       </c>
       <c r="I154" s="4" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J154" s="4" t="n">
         <v>37</v>
       </c>
       <c r="K154" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L154" s="4" t="inlineStr">
         <is>
@@ -16529,11 +16522,11 @@
         </is>
       </c>
       <c r="M154" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N154" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O154" s="7" t="inlineStr">
@@ -16542,7 +16535,7 @@
         </is>
       </c>
       <c r="P154" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q154" s="9" t="n">
         <v>1</v>
@@ -16560,19 +16553,19 @@
         <v>2</v>
       </c>
       <c r="V154" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W154" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X154" s="9" t="n">
-        <v>3</v>
+      <c r="X154" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="Y154" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z154" s="9" t="n">
-        <v>0</v>
+      <c r="Z154" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA154" s="10" t="n">
         <v>1</v>
@@ -16634,11 +16627,11 @@
         </is>
       </c>
       <c r="M155" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N155" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O155" s="7" t="inlineStr">
@@ -16670,8 +16663,8 @@
       <c r="W155" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X155" s="9" t="n">
-        <v>3</v>
+      <c r="X155" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y155" s="9" t="n">
         <v>0</v>
@@ -16772,7 +16765,7 @@
         <v>0</v>
       </c>
       <c r="X156" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y156" s="9" t="n">
         <v>0</v>
@@ -16945,11 +16938,11 @@
         </is>
       </c>
       <c r="M158" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N158" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O158" s="7" t="inlineStr">
@@ -16981,8 +16974,8 @@
       <c r="W158" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X158" s="9" t="n">
-        <v>2</v>
+      <c r="X158" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y158" s="9" t="n">
         <v>0</v>
@@ -17083,7 +17076,7 @@
         <v>0</v>
       </c>
       <c r="X159" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Y159" s="9" t="n">
         <v>0</v>
@@ -17158,9 +17151,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O160" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O160" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P160" s="9" t="n">
@@ -17173,7 +17166,7 @@
         <v>0</v>
       </c>
       <c r="S160" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T160" s="9" t="n">
         <v>0</v>
@@ -17188,7 +17181,7 @@
         <v>0</v>
       </c>
       <c r="X160" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y160" s="9" t="n">
         <v>0</v>
@@ -17242,13 +17235,13 @@
         </is>
       </c>
       <c r="I161" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J161" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K161" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L161" s="4" t="inlineStr">
         <is>
@@ -17287,7 +17280,7 @@
         <v>0</v>
       </c>
       <c r="V161" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W161" s="9" t="n">
         <v>0</v>
@@ -17448,13 +17441,13 @@
         </is>
       </c>
       <c r="I163" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J163" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K163" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L163" s="7" t="inlineStr">
         <is>
@@ -17462,16 +17455,16 @@
         </is>
       </c>
       <c r="M163" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N163" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
-        </is>
-      </c>
-      <c r="O163" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+          <t>Officer list on time</t>
+        </is>
+      </c>
+      <c r="O163" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P163" s="9" t="n">
@@ -17493,13 +17486,13 @@
         <v>0</v>
       </c>
       <c r="V163" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W163" s="9" t="n">
         <v>0</v>
       </c>
       <c r="X163" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y163" s="9" t="n">
         <v>0</v>
@@ -17563,16 +17556,16 @@
         </is>
       </c>
       <c r="M164" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N164" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
-        </is>
-      </c>
-      <c r="O164" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+          <t>Officers trained Nov-Feb</t>
+        </is>
+      </c>
+      <c r="O164" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P164" s="9" t="n">
@@ -17701,7 +17694,7 @@
         <v>0</v>
       </c>
       <c r="X165" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y165" s="9" t="n">
         <v>0</v>
@@ -17765,11 +17758,11 @@
         </is>
       </c>
       <c r="M166" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N166" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O166" s="4" t="inlineStr">
@@ -17801,8 +17794,8 @@
       <c r="W166" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X166" s="9" t="n">
-        <v>3</v>
+      <c r="X166" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y166" s="9" t="n">
         <v>0</v>
@@ -17975,11 +17968,11 @@
         </is>
       </c>
       <c r="M168" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N168" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O168" s="4" t="inlineStr">
@@ -18012,7 +18005,7 @@
         <v>0</v>
       </c>
       <c r="X168" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y168" s="9" t="n">
         <v>0</v>
@@ -18083,9 +18076,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O169" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O169" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P169" s="9" t="n">
@@ -18214,7 +18207,7 @@
         <v>0</v>
       </c>
       <c r="X170" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y170" s="9" t="n">
         <v>0</v>
@@ -18278,11 +18271,11 @@
         </is>
       </c>
       <c r="M171" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N171" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O171" s="7" t="inlineStr">
@@ -18315,7 +18308,7 @@
         <v>0</v>
       </c>
       <c r="X171" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y171" s="9" t="n">
         <v>0</v>
@@ -18379,11 +18372,11 @@
         </is>
       </c>
       <c r="M172" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N172" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O172" s="7" t="inlineStr">
@@ -18415,8 +18408,8 @@
       <c r="W172" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X172" s="9" t="n">
-        <v>3</v>
+      <c r="X172" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y172" s="9" t="n">
         <v>0</v>
@@ -18480,11 +18473,11 @@
         </is>
       </c>
       <c r="M173" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N173" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O173" s="4" t="inlineStr">
@@ -18516,8 +18509,8 @@
       <c r="W173" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X173" s="9" t="n">
-        <v>3</v>
+      <c r="X173" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Y173" s="9" t="n">
         <v>0</v>
@@ -18622,7 +18615,7 @@
         <v>0</v>
       </c>
       <c r="X174" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y174" s="9" t="n">
         <v>0</v>
@@ -18690,11 +18683,11 @@
         </is>
       </c>
       <c r="M175" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N175" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O175" s="4" t="inlineStr">
@@ -18791,11 +18784,11 @@
         </is>
       </c>
       <c r="M176" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N176" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O176" s="7" t="inlineStr">
@@ -19001,11 +18994,11 @@
         </is>
       </c>
       <c r="M178" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N178" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O178" s="7" t="inlineStr">
@@ -19037,8 +19030,8 @@
       <c r="W178" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X178" s="9" t="n">
-        <v>3</v>
+      <c r="X178" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y178" s="9" t="n">
         <v>0</v>
@@ -19211,11 +19204,11 @@
         </is>
       </c>
       <c r="M180" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N180" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O180" s="7" t="inlineStr">
@@ -19248,7 +19241,7 @@
         <v>0</v>
       </c>
       <c r="X180" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y180" s="9" t="n">
         <v>0</v>
@@ -19312,11 +19305,11 @@
         </is>
       </c>
       <c r="M181" s="8" t="n">
-        <v>46265</v>
+        <v>46446</v>
       </c>
       <c r="N181" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officers trained Nov-Feb</t>
         </is>
       </c>
       <c r="O181" s="7" t="inlineStr">
@@ -19413,11 +19406,11 @@
         </is>
       </c>
       <c r="M182" s="8" t="n">
-        <v>46265</v>
+        <v>46387</v>
       </c>
       <c r="N182" s="4" t="inlineStr">
         <is>
-          <t>Officers trained Jun-Aug</t>
+          <t>Officer list on time</t>
         </is>
       </c>
       <c r="O182" s="7" t="inlineStr">
@@ -19554,7 +19547,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -19566,7 +19559,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>2</v>
@@ -19599,7 +19592,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -19632,7 +19625,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
@@ -19665,7 +19658,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
@@ -19698,7 +19691,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
@@ -19731,7 +19724,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -19764,7 +19757,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
@@ -19785,7 +19778,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -19797,7 +19790,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -19830,7 +19823,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
         <v>2</v>
@@ -19863,7 +19856,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -19896,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>2</v>
@@ -19917,7 +19910,7 @@
         <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -19929,7 +19922,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>3</v>
@@ -19962,7 +19955,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
@@ -19995,7 +19988,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
         <v>1</v>
@@ -20028,7 +20021,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>1</v>
@@ -20049,7 +20042,7 @@
         <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -20061,7 +20054,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>3</v>
@@ -20094,7 +20087,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
         <v>2</v>
@@ -20127,7 +20120,7 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
         <v>3</v>
@@ -20226,7 +20219,7 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
         <v>2</v>
@@ -20259,7 +20252,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -20292,7 +20285,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>3</v>
@@ -20325,7 +20318,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>2</v>
@@ -20391,7 +20384,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -20424,7 +20417,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>2</v>
@@ -20457,7 +20450,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
         <v>3</v>
@@ -20490,7 +20483,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
         <v>2</v>
@@ -20511,7 +20504,7 @@
         <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
@@ -20556,7 +20549,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
         <v>1</v>
@@ -20577,7 +20570,7 @@
         <v>5</v>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
@@ -20589,7 +20582,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>3</v>
@@ -20622,7 +20615,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>2</v>
@@ -20688,7 +20681,7 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -20721,7 +20714,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>1</v>
@@ -20754,7 +20747,7 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
         <v>2</v>
@@ -20787,7 +20780,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
         <v>1</v>

</xml_diff>